<commit_message>
feat(F-NAR-019): TREE-AUT-038 polish Le seau sous la table
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-038.xlsx
+++ b/stories/arbres/TREE-AUT-038.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le bois de la table fait tic au soleil. Il sèche, sans personne. Un pain tiède y pose son ventre. Ça sent la croûte, près du nez. Une mouche marche sur la mie. Mila pose sa joue sur le bois. Il est chaud, maman. Le pain vient du fournil. Un seau jaune attend près du pied. L'anse a un clou de cuivre. Le clou cligne, une fois. Tu as vu ce clou, Mila ? Il brille, papa. En ce moment, Mila veut le bac. Un gâteau de sable, vite ! Elle tire le seau par l'anse. Un pigeon se pose sur le pain. Il pique une miette, nette. Oh ! Mila sursaute. Le seau roule sous la table. Toc, contre le pied de bois. Le clou de cuivre s'éteint, à l'ombre. Il reste là, à l'abri. On y va ? Mila pousse le seau plus loin. Il ne roule plus. Elle part, les mains vides.</t>
+          <t>Le bois de la table fait tic au soleil. Il sèche, sans personne. Un pain tiède y pose son ventre. Ça sent la croûte, près du nez. Une mouche marche sur la mie. Mila pose sa joue sur le bois. Il est chaud, maman. Le pain vient du fournil. Un seau jaune attend près du pied. L'anse a un clou de cuivre. Le clou cligne, une fois. Tu as vu ce clou, Mila ? Il brille, papa. En ce moment, Mila veut le bac. Un gâteau de sable, vite ! Elle tire le seau par l'anse. Un pigeon se pose sur le pain. Il pique une miette, nette. Oh ! Mila sursaute. Le seau roule sous la table. Toc, contre le pied de bois. Le clou de cuivre s'éteint, à l'ombre. Une miette reste collée à l'anse. Il reste là, à l'abri. On y va ? Mila pousse le seau plus loin. Il ne roule plus. Elle part, les mains vides.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le bois de la table fait tic au soleil. Il sèche, sans personne. Un pain tiède y pose son ventre. Ça sent la croûte, près du nez. Une mouche marche sur la mie. Mila pose sa joue sur le bois. Il est chaud, maman. Le pain vient du fournil. Un seau jaune attend près du pied. L'anse a un &lt;emphasis level="moderate"&gt;clou de cuivre&lt;/emphasis&gt;. Le clou cligne, une fois. Tu as vu ce clou, Mila ? Il brille, papa. En ce moment, Mila veut le bac. Un gâteau de sable, vite ! Elle tire le seau par l'anse. Un pigeon se pose sur le pain. Il pique une miette, nette. Oh ! Mila sursaute. Le seau roule sous la table. Toc, contre le pied de bois. Le clou de cuivre s'éteint, à l'ombre. Il reste là, à l'abri. On y va ? Mila pousse le seau plus loin. Il ne roule plus. Elle part, les mains vides.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le bois de la table fait tic au soleil. Il sèche, sans personne. Un pain tiède y pose son ventre. Ça sent la croûte, près du nez. Une mouche marche sur la mie. Mila pose sa joue sur le bois. Il est chaud, maman. Le pain vient du fournil. Un seau jaune attend près du pied. L'anse a un &lt;emphasis level="moderate"&gt;clou de cuivre&lt;/emphasis&gt;. Le clou cligne, une fois. Tu as vu ce clou, Mila ? Il brille, papa. En ce moment, Mila veut le bac. Un gâteau de sable, vite ! Elle tire le seau par l'anse. Un pigeon se pose sur le pain. Il pique une miette, nette. Oh ! Mila sursaute. Le seau roule sous la table. Toc, contre le pied de bois. Le clou de cuivre s'éteint, à l'ombre. Une miette reste collée à l'anse. Il reste là, à l'abri. On y va ? Mila pousse le seau plus loin. Il ne roule plus. Elle part, les mains vides.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le bois de la table fait tic au soleil. Il sèche, sans personne. Un pain tiède y pose son ventre. Ça sent la croûte, près du nez. Une mouche marche sur la mie. Mila pose sa joue sur le bois. Il est chaud, maman. Le pain vient du fournil. Un seau jaune attend près du pied. L'anse a un &lt;emphasis&gt;clou de cuivre&lt;/emphasis&gt;. Le clou cligne, une fois. Tu as vu ce clou, Mila ? Il brille, papa. En ce moment, Mila veut le bac. Un gâteau de sable, vite ! Elle tire le seau par l'anse. Un pigeon se pose sur le pain. Il pique une miette, nette. Oh ! Mila sursaute. Le seau roule sous la table. Toc, contre le pied de bois. Le clou de cuivre s'éteint, à l'ombre. Il reste là, à l'abri. On y va ? Mila pousse le seau plus loin. Il ne roule plus. Elle part, les mains vides. [pause]</t>
+          <t>Le bois de la table fait tic au soleil. Il sèche, sans personne. Un pain tiède y pose son ventre. Ça sent la croûte, près du nez. Une mouche marche sur la mie. Mila pose sa joue sur le bois. Il est chaud, maman. Le pain vient du fournil. Un seau jaune attend près du pied. L'anse a un &lt;emphasis&gt;clou de cuivre&lt;/emphasis&gt;. Le clou cligne, une fois. Tu as vu ce clou, Mila ? Il brille, papa. En ce moment, Mila veut le bac. Un gâteau de sable, vite ! Elle tire le seau par l'anse. Un pigeon se pose sur le pain. Il pique une miette, nette. Oh ! Mila sursaute. Le seau roule sous la table. Toc, contre le pied de bois. Le clou de cuivre s'éteint, à l'ombre. Une miette reste collée à l'anse. Il reste là, à l'abri. On y va ? Mila pousse le seau plus loin. Il ne roule plus. Elle part, les mains vides. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1364,6 +1364,7 @@
 narrateur|Le seau roule sous la table.
 narrateur|Toc, contre le pied de bois.
 narrateur|Le clou de cuivre s'éteint, à l'ombre.
+narrateur|Une miette reste collée à l'anse.
 enfant-f|Il reste là, à l'abri.
 papa|On y va ?
 narrateur|Mila pousse le seau plus loin.
@@ -1603,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila s'agenouille près du bac. Le sable est frais, un peu fin. Il coule entre ses doigts. Un gâteau, maman. Avec tes mains ? Avec le seau ! Elle court vers la table. Elle tire l'anse, trop fort. L'anse bute contre le pied. Il ne vient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il est où ? Tu l'as vu, au départ.</t>
+          <t>Mila s'agenouille près du bac. Le sable est frais, un peu fin. Il coule entre ses doigts. Un gâteau, maman. Avec tes mains ? Avec le seau ! Elle court vers la table. Elle tire l'anse, trop fort. L'anse bute contre le pied. Le seau recule, dans l'ombre. Il ne vient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il est où ? Tu l'as vu, au départ.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila s'agenouille près du bac. Le sable est frais, un peu fin. Il coule entre ses doigts. Un &lt;emphasis level="moderate"&gt;gâteau&lt;/emphasis&gt;, maman. Avec tes mains ? Avec le seau ! Elle court vers la table. Elle tire l'anse, trop fort. L'anse bute contre le pied. Il ne vient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il est où ? Tu l'as vu, au départ.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila s'agenouille près du bac. Le sable est frais, un peu fin. Il coule entre ses doigts. Un &lt;emphasis level="moderate"&gt;gâteau&lt;/emphasis&gt;, maman. Avec tes mains ? Avec le seau ! Elle court vers la table. Elle tire l'anse, trop fort. L'anse bute contre le pied. Le seau recule, dans l'ombre. Il ne vient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il est où ? Tu l'as vu, au départ.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Mila s'agenouille près du bac. Le sable est frais, un peu fin. Il coule entre ses doigts. Un &lt;emphasis&gt;gâteau&lt;/emphasis&gt;, maman. Avec tes mains ? Avec le seau ! Elle court vers la table. Elle tire l'anse, trop fort. L'anse bute contre le pied. Il ne vient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il est où ? Tu l'as vu, au départ. [pause]</t>
+          <t>Mila s'agenouille près du bac. Le sable est frais, un peu fin. Il coule entre ses doigts. Un &lt;emphasis&gt;gâteau&lt;/emphasis&gt;, maman. Avec tes mains ? Avec le seau ! Elle court vers la table. Elle tire l'anse, trop fort. L'anse bute contre le pied. Le seau recule, dans l'ombre. Il ne vient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il est où ? Tu l'as vu, au départ. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1756,6 +1757,7 @@
 narrateur|Elle court vers la table.
 narrateur|Elle tire l'anse, trop fort.
 narrateur|L'anse bute contre le pied.
+narrateur|Le seau recule, dans l'ombre.
 enfant-f|Il ne vient pas.
 narrateur|Le sourire de Mila disparaît.
 narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
@@ -2363,17 +2365,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, le ballon rouge attend. Il est lisse, un peu frais. Il pousse le sable ! Mila frappe trop fort. Le ballon file sous la table. Le seau aussi ? Elle se jette à plat ventre. Sa main trouve le cuir rouge. Pas l'anse. Ce n'est pas lui. La serviette du pain tombe, large. Elle cache le clou de cuivre. On tire tout ? Non. Mila refuse de foncer. Elle écoute le square. Toc, très loin, sous le bois. Le clou. Tu l'as entendu, toi.</t>
+          <t>Près du bac, le ballon rouge attend. Il est lisse, un peu frais. Il pousse le sable ! Mila frappe trop fort. Le ballon file sous la table. Le seau aussi ? Elle se jette à plat ventre. Sa main trouve le cuir rouge. Pas l'anse. Ce n'est pas lui. La serviette du pain tombe, large. Elle cache le clou de cuivre. On tire tout ? Non. Mila refuse de foncer. Elle écoute le square. Le pigeon reprend une miette, loin. C'est l'heure, presque. Pas sans le toc. Toc, très loin, sous le bois. Le clou. Tu l'as entendu, toi.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près du bac, le ballon rouge attend. Il est lisse, un peu frais. Il pousse le sable ! Mila frappe trop fort. Le ballon file sous la table. Le seau aussi ? Elle se jette à plat ventre. Sa main trouve le cuir rouge. Pas l'anse. Ce n'est pas lui. La serviette du pain tombe, large. Elle cache le clou de cuivre. On tire tout ? Non. Mila refuse de foncer. Elle écoute le square. Toc, très loin, sous le bois. Le clou. Tu l'as entendu, toi.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près du bac, le ballon rouge attend. Il est lisse, un peu frais. Il pousse le sable ! Mila frappe trop fort. Le ballon file sous la table. Le seau aussi ? Elle se jette à plat ventre. Sa main trouve le cuir rouge. Pas l'anse. Ce n'est pas lui. La serviette du pain tombe, large. Elle cache le clou de cuivre. On tire tout ? Non. Mila refuse de foncer. Elle écoute le square. Le pigeon reprend une miette, loin. C'est l'heure, presque. Pas sans le toc. Toc, très loin, sous le bois. Le clou. Tu l'as entendu, toi.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Près du bac, le ballon rouge attend. Il est lisse, un peu frais. Il pousse le sable ! Mila frappe trop fort. Le ballon file sous la table. Le seau aussi ? Elle se jette à plat ventre. Sa main trouve le cuir rouge. Pas l'anse. Ce n'est pas lui. La serviette du pain tombe, large. Elle cache le clou de cuivre. On tire tout ? Non. Mila refuse de foncer. Elle écoute le square. Toc, très loin, sous le bois. Le clou. Tu l'as entendu, toi.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Près du bac, le ballon rouge attend. Il est lisse, un peu frais. Il pousse le sable ! Mila frappe trop fort. Le ballon file sous la table. Le seau aussi ? Elle se jette à plat ventre. Sa main trouve le cuir rouge. Pas l'anse. Ce n'est pas lui. La serviette du pain tombe, large. Elle cache le clou de cuivre. On tire tout ? Non. Mila refuse de foncer. Elle écoute le square. Le pigeon reprend une miette, loin. C'est l'heure, presque. Pas sans le toc. Toc, très loin, sous le bois. Le clou. Tu l'as entendu, toi.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2527,6 +2529,9 @@
 enfant-f|Non.
 narrateur|Mila refuse de foncer.
 narrateur|Elle écoute le square.
+narrateur|Le pigeon reprend une miette, loin.
+papa|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 narrateur|Toc, très loin, sous le bois.
 enfant-f|Le clou.
 maman|Tu l'as entendu, toi.</t>
@@ -3899,17 +3904,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Mila revient vers la table. L'ombre sous le plateau est froide. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute, sèche, contre le pied. Il reste. La serviette glisse du pain. Elle tombe comme un rideau. Le clou de cuivre disparaît. Je n'aime pas ça. On s'accroupit ? Maman se met à sa hauteur. Je tire, moi ? Non. Mila refuse de foncer. Elle observe le seau, dans le noir. Elle écoute le bois. Le toc du clou. Tu l'as, ce son.</t>
+          <t>Mila revient vers la table. L'ombre sous le plateau est froide. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute, sèche, contre le pied. Il reste. La serviette glisse du pain. Elle tombe comme un rideau. Le clou de cuivre disparaît. Je n'aime pas ça. On s'accroupit ? Maman se met à sa hauteur. Je tire, moi ? Non. Mila refuse de foncer. Elle observe le seau, dans le noir. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce son.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila revient vers la table. L'ombre sous le plateau est froide. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute, sèche, contre le pied. Il reste. La serviette glisse du pain. Elle tombe comme un rideau. Le clou de cuivre disparaît. Je n'aime pas ça. On s'accroupit ? Maman se met à sa hauteur. Je tire, moi ? Non. Mila refuse de foncer. Elle observe le seau, dans le noir. Elle écoute le bois. Le toc du clou. Tu l'as, ce son.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila revient vers la table. L'ombre sous le plateau est froide. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute, sèche, contre le pied. Il reste. La serviette glisse du pain. Elle tombe comme un rideau. Le clou de cuivre disparaît. Je n'aime pas ça. On s'accroupit ? Maman se met à sa hauteur. Je tire, moi ? Non. Mila refuse de foncer. Elle observe le seau, dans le noir. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce son.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Mila revient vers la table. L'ombre sous le plateau est froide. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute, sèche, contre le pied. Il reste. La serviette glisse du pain. Elle tombe comme un rideau. Le clou de cuivre disparaît. Je n'aime pas ça. On s'accroupit ? Maman se met à sa hauteur. Je tire, moi ? Non. Mila refuse de foncer. Elle observe le seau, dans le noir. Elle écoute le bois. Le toc du clou. Tu l'as, ce son.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Mila revient vers la table. L'ombre sous le plateau est froide. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute, sèche, contre le pied. Il reste. La serviette glisse du pain. Elle tombe comme un rideau. Le clou de cuivre disparaît. Je n'aime pas ça. On s'accroupit ? Maman se met à sa hauteur. Je tire, moi ? Non. Mila refuse de foncer. Elle observe le seau, dans le noir. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce son.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -4064,6 +4069,8 @@
 narrateur|Mila refuse de foncer.
 narrateur|Elle observe le seau, dans le noir.
 narrateur|Elle écoute le bois.
+papa|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 enfant-f|Le toc du clou.
 papa|Tu l'as, ce son.</t>
         </is>
@@ -5431,17 +5438,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Près du bac, le doudou gris attend. Le tissu est chaud, un peu lourd. Il voit sous la table. Mila le serre trop fort. L'oreille grise cache l'ombre. Elle cherche l'anse, à l'aveugle. Sa main trouve le banc, pas le seau. Il n'est pas là. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. Un grain colle à l'oreille grise.</t>
+          <t>Près du bac, le doudou gris attend. Le tissu est chaud, un peu lourd. Il voit sous la table. Mila le serre trop fort. L'oreille grise cache l'ombre. Elle cherche l'anse, à l'aveugle. Sa main trouve le banc, pas le seau. Il n'est pas là. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. Un grain colle à l'oreille grise.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près du bac, le doudou gris attend. Le tissu est chaud, un peu lourd. Il voit sous la table. Mila le serre trop fort. L'oreille grise cache l'ombre. Elle cherche l'anse, à l'aveugle. Sa main trouve le banc, pas le seau. Il n'est pas là. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. Un grain colle à l'oreille grise.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près du bac, le doudou gris attend. Le tissu est chaud, un peu lourd. Il voit sous la table. Mila le serre trop fort. L'oreille grise cache l'ombre. Elle cherche l'anse, à l'aveugle. Sa main trouve le banc, pas le seau. Il n'est pas là. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. Un grain colle à l'oreille grise.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Près du bac, le doudou gris attend. Le tissu est chaud, un peu lourd. Il voit sous la table. Mila le serre trop fort. L'oreille grise cache l'ombre. Elle cherche l'anse, à l'aveugle. Sa main trouve le banc, pas le seau. Il n'est pas là. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. Un grain colle à l'oreille grise.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Près du bac, le doudou gris attend. Le tissu est chaud, un peu lourd. Il voit sous la table. Mila le serre trop fort. L'oreille grise cache l'ombre. Elle cherche l'anse, à l'aveugle. Sa main trouve le banc, pas le seau. Il n'est pas là. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. Un grain colle à l'oreille grise.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5593,6 +5600,8 @@
 enfant-f|J'attends.
 narrateur|Mila refuse de foncer.
 narrateur|Elle écarte l'oreille, lentement.
+papa|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 narrateur|Un toc minuscule, sous le bois.
 enfant-f|Le clou.
 maman|Tu l'as entendu, seule.
@@ -6958,17 +6967,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Mila grimpe la marche du toboggan. Le plastique est lisse, un peu froid. Une miette de pain y colle. Le seau glisse avec moi ! Il est où, ce seau ? Je le prends. Elle redescend, trop vite. Elle tire l'anse sous le bois. L'anse bute, sèche. Zut. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je m'accroupis, d'accord ? Maman se met à sa hauteur. Le clou ne cligne plus. Tu l'as vu, toi.</t>
+          <t>Mila grimpe la marche du toboggan. Le plastique est lisse, un peu froid. Une miette de pain y colle. Le seau glisse avec moi ! Il est où, ce seau ? Je le prends. Elle redescend, trop vite. Elle tire l'anse sous le bois. L'anse bute, sèche. Le seau recule, dans l'ombre. Zut. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je m'accroupis, d'accord ? Maman se met à sa hauteur. Le clou ne cligne plus. Tu l'as vu, toi.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila grimpe la marche du toboggan. Le plastique est lisse, un peu froid. Une miette de pain y colle. Le seau glisse avec moi ! Il est où, ce seau ? Je le prends. Elle redescend, trop vite. Elle tire l'anse sous le bois. L'anse bute, sèche. Zut. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je m'accroupis, d'accord ? Maman se met à sa hauteur. Le clou ne cligne plus. Tu l'as vu, toi.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila grimpe la marche du toboggan. Le plastique est lisse, un peu froid. Une miette de pain y colle. Le seau glisse avec moi ! Il est où, ce seau ? Je le prends. Elle redescend, trop vite. Elle tire l'anse sous le bois. L'anse bute, sèche. Le seau recule, dans l'ombre. Zut. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je m'accroupis, d'accord ? Maman se met à sa hauteur. Le clou ne cligne plus. Tu l'as vu, toi.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Mila grimpe la marche du toboggan. Le plastique est lisse, un peu froid. Une miette de pain y colle. Le seau glisse avec moi ! Il est où, ce seau ? Je le prends. Elle redescend, trop vite. Elle tire l'anse sous le bois. L'anse bute, sèche. Zut. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je m'accroupis, d'accord ? Maman se met à sa hauteur. Le clou ne cligne plus. Tu l'as vu, toi. [pause]</t>
+          <t>Mila grimpe la marche du toboggan. Le plastique est lisse, un peu froid. Une miette de pain y colle. Le seau glisse avec moi ! Il est où, ce seau ? Je le prends. Elle redescend, trop vite. Elle tire l'anse sous le bois. L'anse bute, sèche. Le seau recule, dans l'ombre. Zut. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je m'accroupis, d'accord ? Maman se met à sa hauteur. Le clou ne cligne plus. Tu l'as vu, toi. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -7111,6 +7120,7 @@
 narrateur|Elle redescend, trop vite.
 narrateur|Elle tire l'anse sous le bois.
 narrateur|L'anse bute, sèche.
+narrateur|Le seau recule, dans l'ombre.
 enfant-f|Zut.
 narrateur|Le sourire de Mila disparaît.
 narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
@@ -7718,17 +7728,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Au pied du toboggan, le ballon attend. Il est froid, près de la rampe. Il roule jusqu'au seau ! Mila le lance trop fort. Le ballon tape le pied de table. Il rebondit, puis se cache. Avec le seau ? Elle rampe. Sa main attrape le cuir, pas l'anse. Faux. Une miette de marche tombe, large. Elle colle au clou de cuivre. On chasse tout ? Non. Mila refuse de foncer. Elle écoute le square. Toc, sous le plastique et le bois. Le clou est là. Tu l'as trouvé, ce son.</t>
+          <t>Au pied du toboggan, le ballon attend. Il est froid, près de la rampe. Il roule jusqu'au seau ! Mila le lance trop fort. Le ballon tape le pied de table. Il rebondit, puis se cache. Avec le seau ? Elle rampe. Sa main attrape le cuir, pas l'anse. Faux. Une miette de marche tombe, large. Elle colle au clou de cuivre. On chasse tout ? Non. Mila refuse de foncer. Elle écoute le square. C'est l'heure, presque. Pas sans le toc. Toc, sous le plastique et le bois. Le clou est là. Tu l'as trouvé, ce son.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au pied du toboggan, le ballon attend. Il est froid, près de la rampe. Il roule jusqu'au seau ! Mila le lance trop fort. Le ballon tape le pied de table. Il rebondit, puis se cache. Avec le seau ? Elle rampe. Sa main attrape le cuir, pas l'anse. Faux. Une miette de marche tombe, large. Elle colle au clou de cuivre. On chasse tout ? Non. Mila refuse de foncer. Elle écoute le square. Toc, sous le plastique et le bois. Le clou est là. Tu l'as trouvé, ce son.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au pied du toboggan, le ballon attend. Il est froid, près de la rampe. Il roule jusqu'au seau ! Mila le lance trop fort. Le ballon tape le pied de table. Il rebondit, puis se cache. Avec le seau ? Elle rampe. Sa main attrape le cuir, pas l'anse. Faux. Une miette de marche tombe, large. Elle colle au clou de cuivre. On chasse tout ? Non. Mila refuse de foncer. Elle écoute le square. C'est l'heure, presque. Pas sans le toc. Toc, sous le plastique et le bois. Le clou est là. Tu l'as trouvé, ce son.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Au pied du toboggan, le ballon attend. Il est froid, près de la rampe. Il roule jusqu'au seau ! Mila le lance trop fort. Le ballon tape le pied de table. Il rebondit, puis se cache. Avec le seau ? Elle rampe. Sa main attrape le cuir, pas l'anse. Faux. Une miette de marche tombe, large. Elle colle au clou de cuivre. On chasse tout ? Non. Mila refuse de foncer. Elle écoute le square. Toc, sous le plastique et le bois. Le clou est là. Tu l'as trouvé, ce son.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Au pied du toboggan, le ballon attend. Il est froid, près de la rampe. Il roule jusqu'au seau ! Mila le lance trop fort. Le ballon tape le pied de table. Il rebondit, puis se cache. Avec le seau ? Elle rampe. Sa main attrape le cuir, pas l'anse. Faux. Une miette de marche tombe, large. Elle colle au clou de cuivre. On chasse tout ? Non. Mila refuse de foncer. Elle écoute le square. C'est l'heure, presque. Pas sans le toc. Toc, sous le plastique et le bois. Le clou est là. Tu l'as trouvé, ce son.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7882,6 +7892,8 @@
 enfant-f|Non.
 narrateur|Mila refuse de foncer.
 narrateur|Elle écoute le square.
+maman|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 narrateur|Toc, sous le plastique et le bois.
 enfant-f|Le clou est là.
 papa|Tu l'as trouvé, ce son.</t>
@@ -9248,17 +9260,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Mila revient vers la table. Une miette brille sur la marche. Le seau, papa. Elle tire, trop vite. L'anse bute, sèche. Le seau penche, puis recule. Il ne veut pas. La serviette du pain tombe. Elle cache le clou de cuivre. Un coup sec ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le lieu. Mila observe le seau, dans l'ombre. Elle écoute le bois. Le toc du clou. Tu l'as, ce bruit. La miette reste sur le plastique.</t>
+          <t>Mila revient vers la table. Une miette brille sur la marche. Le seau, papa. Elle tire, trop vite. L'anse bute, sèche. Le seau penche, puis recule. Il ne veut pas. La serviette du pain tombe. Elle cache le clou de cuivre. Un coup sec ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le lieu. Mila observe le seau, dans l'ombre. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce bruit. La miette reste sur le plastique.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila revient vers la table. Une miette brille sur la marche. Le seau, papa. Elle tire, trop vite. L'anse bute, sèche. Le seau penche, puis recule. Il ne veut pas. La serviette du pain tombe. Elle cache le clou de cuivre. Un coup sec ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le lieu. Mila observe le seau, dans l'ombre. Elle écoute le bois. Le toc du clou. Tu l'as, ce bruit. La miette reste sur le plastique.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila revient vers la table. Une miette brille sur la marche. Le seau, papa. Elle tire, trop vite. L'anse bute, sèche. Le seau penche, puis recule. Il ne veut pas. La serviette du pain tombe. Elle cache le clou de cuivre. Un coup sec ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le lieu. Mila observe le seau, dans l'ombre. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce bruit. La miette reste sur le plastique.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Mila revient vers la table. Une miette brille sur la marche. Le seau, papa. Elle tire, trop vite. L'anse bute, sèche. Le seau penche, puis recule. Il ne veut pas. La serviette du pain tombe. Elle cache le clou de cuivre. Un coup sec ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le lieu. Mila observe le seau, dans l'ombre. Elle écoute le bois. Le toc du clou. Tu l'as, ce bruit. La miette reste sur le plastique.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Mila revient vers la table. Une miette brille sur la marche. Le seau, papa. Elle tire, trop vite. L'anse bute, sèche. Le seau penche, puis recule. Il ne veut pas. La serviette du pain tombe. Elle cache le clou de cuivre. Un coup sec ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le lieu. Mila observe le seau, dans l'ombre. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce bruit. La miette reste sur le plastique.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9412,6 +9424,8 @@
 narrateur|Personne ne dit le lieu.
 narrateur|Mila observe le seau, dans l'ombre.
 narrateur|Elle écoute le bois.
+papa|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 enfant-f|Le toc du clou.
 maman|Tu l'as, ce bruit.
 narrateur|La miette reste sur le plastique.</t>
@@ -10778,17 +10792,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Au toboggan, le doudou a vu la rampe. L'oreille grise est un peu froide. Il attrape le seau, en bas. Mila glisse le doudou sous le bois. Le tissu s'accroche au pied. L'anse reste loin. Il est coincé, lui. Le sourire de Mila disparaît. On tire le tissu ? Doucement. Mila refuse de foncer. Elle recule le doudou, un pouce. Puis un autre. Un toc minuscule, sous le plateau. Le clou. Tu l'as entendu, seule. Papa se met à sa hauteur. Une miette colle au ventre gris.</t>
+          <t>Au toboggan, le doudou a vu la rampe. L'oreille grise est un peu froide. Il attrape le seau, en bas. Mila glisse le doudou sous le bois. Le tissu s'accroche au pied. L'anse reste loin. Il est coincé, lui. Le sourire de Mila disparaît. On tire le tissu ? Doucement. Mila refuse de foncer. Elle recule le doudou, un pouce. Puis un autre. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le plateau. Le clou. Tu l'as entendu, seule. Papa se met à sa hauteur. Une miette colle au ventre gris.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au toboggan, le doudou a vu la rampe. L'oreille grise est un peu froide. Il attrape le seau, en bas. Mila glisse le doudou sous le bois. Le tissu s'accroche au pied. L'anse reste loin. Il est coincé, lui. Le sourire de Mila disparaît. On tire le tissu ? Doucement. Mila refuse de foncer. Elle recule le doudou, un pouce. Puis un autre. Un toc minuscule, sous le plateau. Le clou. Tu l'as entendu, seule. Papa se met à sa hauteur. Une miette colle au ventre gris.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au toboggan, le doudou a vu la rampe. L'oreille grise est un peu froide. Il attrape le seau, en bas. Mila glisse le doudou sous le bois. Le tissu s'accroche au pied. L'anse reste loin. Il est coincé, lui. Le sourire de Mila disparaît. On tire le tissu ? Doucement. Mila refuse de foncer. Elle recule le doudou, un pouce. Puis un autre. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le plateau. Le clou. Tu l'as entendu, seule. Papa se met à sa hauteur. Une miette colle au ventre gris.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Au toboggan, le doudou a vu la rampe. L'oreille grise est un peu froide. Il attrape le seau, en bas. Mila glisse le doudou sous le bois. Le tissu s'accroche au pied. L'anse reste loin. Il est coincé, lui. Le sourire de Mila disparaît. On tire le tissu ? Doucement. Mila refuse de foncer. Elle recule le doudou, un pouce. Puis un autre. Un toc minuscule, sous le plateau. Le clou. Tu l'as entendu, seule. Papa se met à sa hauteur. Une miette colle au ventre gris.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Au toboggan, le doudou a vu la rampe. L'oreille grise est un peu froide. Il attrape le seau, en bas. Mila glisse le doudou sous le bois. Le tissu s'accroche au pied. L'anse reste loin. Il est coincé, lui. Le sourire de Mila disparaît. On tire le tissu ? Doucement. Mila refuse de foncer. Elle recule le doudou, un pouce. Puis un autre. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le plateau. Le clou. Tu l'as entendu, seule. Papa se met à sa hauteur. Une miette colle au ventre gris.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10939,6 +10953,8 @@
 narrateur|Mila refuse de foncer.
 narrateur|Elle recule le doudou, un pouce.
 narrateur|Puis un autre.
+papa|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 narrateur|Un toc minuscule, sous le plateau.
 enfant-f|Le clou.
 maman|Tu l'as entendu, seule.
@@ -12305,17 +12321,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Mila va vers les balançoires. Une chaîne fait tic, mince. Le siège rouge est tiède. Le seau s'assoit avec moi. Il est resté où ? Je le cherche. Elle court, les mains ouvertes. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste coincé. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il s'est tu. Tu l'as entendu, au départ.</t>
+          <t>Mila va vers les balançoires. Une chaîne fait tic, mince. Le siège rouge est tiède. Le seau s'assoit avec moi. Il est resté où ? Je le cherche. Elle court, les mains ouvertes. Elle tire l'anse d'un coup. L'anse bute contre le pied. Le seau recule, dans l'ombre. Il reste coincé. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il s'est tu. Tu l'as entendu, au départ.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila va vers les balançoires. Une chaîne fait tic, mince. Le siège rouge est tiède. Le seau s'assoit avec moi. Il est resté où ? Je le cherche. Elle court, les mains ouvertes. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste coincé. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il s'est tu. Tu l'as entendu, au départ.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila va vers les balançoires. Une chaîne fait tic, mince. Le siège rouge est tiède. Le seau s'assoit avec moi. Il est resté où ? Je le cherche. Elle court, les mains ouvertes. Elle tire l'anse d'un coup. L'anse bute contre le pied. Le seau recule, dans l'ombre. Il reste coincé. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il s'est tu. Tu l'as entendu, au départ.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Mila va vers les balançoires. Une chaîne fait tic, mince. Le siège rouge est tiède. Le seau s'assoit avec moi. Il est resté où ? Je le cherche. Elle court, les mains ouvertes. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste coincé. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il s'est tu. Tu l'as entendu, au départ. [pause]</t>
+          <t>Mila va vers les balançoires. Une chaîne fait tic, mince. Le siège rouge est tiède. Le seau s'assoit avec moi. Il est resté où ? Je le cherche. Elle court, les mains ouvertes. Elle tire l'anse d'un coup. L'anse bute contre le pied. Le seau recule, dans l'ombre. Il reste coincé. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On s'accroupit ? Papa se met à sa hauteur. Le clou, il s'est tu. Tu l'as entendu, au départ. [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12458,6 +12474,7 @@
 narrateur|Elle court, les mains ouvertes.
 narrateur|Elle tire l'anse d'un coup.
 narrateur|L'anse bute contre le pied.
+narrateur|Le seau recule, dans l'ombre.
 enfant-f|Il reste coincé.
 narrateur|Le sourire de Mila disparaît.
 narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
@@ -13065,17 +13082,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Près des chaînes, le ballon rouge attend. Il est lisse, un peu frais. Il roule sous la table ! Mila pousse trop fort. Le ballon rebondit une fois, mou. Il se cache derrière le pied. Le seau aussi ? Elle rampe, le vent dans le dos. Sa main trouve le cuir. Pas l'anse jaune. Ce n'est pas lui. On chasse le ballon ? Non. Mila refuse de foncer. Elle écoute le square. La chaîne se tait. Toc, sous le bois, minuscule. Le clou. Tu l'as entendu, toi.</t>
+          <t>Près des chaînes, le ballon rouge attend. Il est lisse, un peu frais. Il roule sous la table ! Mila pousse trop fort. Le ballon rebondit une fois, mou. Il se cache derrière le pied. Le seau aussi ? Elle rampe, le vent dans le dos. Sa main trouve le cuir. Pas l'anse jaune. Ce n'est pas lui. On chasse le ballon ? Non. Mila refuse de foncer. Elle écoute le square. La chaîne se tait. C'est l'heure, presque. Pas sans le toc. Toc, sous le bois, minuscule. Le clou. Tu l'as entendu, toi.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près des chaînes, le ballon rouge attend. Il est lisse, un peu frais. Il roule sous la table ! Mila pousse trop fort. Le ballon rebondit une fois, mou. Il se cache derrière le pied. Le seau aussi ? Elle rampe, le vent dans le dos. Sa main trouve le cuir. Pas l'anse jaune. Ce n'est pas lui. On chasse le ballon ? Non. Mila refuse de foncer. Elle écoute le square. La chaîne se tait. Toc, sous le bois, minuscule. Le clou. Tu l'as entendu, toi.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près des chaînes, le ballon rouge attend. Il est lisse, un peu frais. Il roule sous la table ! Mila pousse trop fort. Le ballon rebondit une fois, mou. Il se cache derrière le pied. Le seau aussi ? Elle rampe, le vent dans le dos. Sa main trouve le cuir. Pas l'anse jaune. Ce n'est pas lui. On chasse le ballon ? Non. Mila refuse de foncer. Elle écoute le square. La chaîne se tait. C'est l'heure, presque. Pas sans le toc. Toc, sous le bois, minuscule. Le clou. Tu l'as entendu, toi.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Près des chaînes, le ballon rouge attend. Il est lisse, un peu frais. Il roule sous la table ! Mila pousse trop fort. Le ballon rebondit une fois, mou. Il se cache derrière le pied. Le seau aussi ? Elle rampe, le vent dans le dos. Sa main trouve le cuir. Pas l'anse jaune. Ce n'est pas lui. On chasse le ballon ? Non. Mila refuse de foncer. Elle écoute le square. La chaîne se tait. Toc, sous le bois, minuscule. Le clou. Tu l'as entendu, toi.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Près des chaînes, le ballon rouge attend. Il est lisse, un peu frais. Il roule sous la table ! Mila pousse trop fort. Le ballon rebondit une fois, mou. Il se cache derrière le pied. Le seau aussi ? Elle rampe, le vent dans le dos. Sa main trouve le cuir. Pas l'anse jaune. Ce n'est pas lui. On chasse le ballon ? Non. Mila refuse de foncer. Elle écoute le square. La chaîne se tait. C'est l'heure, presque. Pas sans le toc. Toc, sous le bois, minuscule. Le clou. Tu l'as entendu, toi.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -13229,6 +13246,8 @@
 narrateur|Mila refuse de foncer.
 narrateur|Elle écoute le square.
 narrateur|La chaîne se tait.
+maman|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 narrateur|Toc, sous le bois, minuscule.
 enfant-f|Le clou.
 papa|Tu l'as entendu, toi.</t>
@@ -14596,17 +14615,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Mila revient vers la table. Le vent a touché le pain. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste. Le manteau rouge bouge au dossier. Une manche tombe, large. Elle cache le clou de cuivre. On soulève tout ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le mot. Mila observe le seau, dans l'ombre. Elle écoute le bois. Le toc du clou. Tu l'as, ce son. La chaîne reste muette, derrière.</t>
+          <t>Mila revient vers la table. Le vent a touché le pain. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste. Le manteau rouge bouge au dossier. Une manche tombe, large. Elle cache le clou de cuivre. On soulève tout ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le mot. Mila observe le seau, dans l'ombre. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce son. La chaîne reste muette, derrière.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila revient vers la table. Le vent a touché le pain. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste. Le manteau rouge bouge au dossier. Une manche tombe, large. Elle cache le clou de cuivre. On soulève tout ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le mot. Mila observe le seau, dans l'ombre. Elle écoute le bois. Le toc du clou. Tu l'as, ce son. La chaîne reste muette, derrière.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila revient vers la table. Le vent a touché le pain. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste. Le manteau rouge bouge au dossier. Une manche tombe, large. Elle cache le clou de cuivre. On soulève tout ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le mot. Mila observe le seau, dans l'ombre. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce son. La chaîne reste muette, derrière.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Mila revient vers la table. Le vent a touché le pain. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste. Le manteau rouge bouge au dossier. Une manche tombe, large. Elle cache le clou de cuivre. On soulève tout ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le mot. Mila observe le seau, dans l'ombre. Elle écoute le bois. Le toc du clou. Tu l'as, ce son. La chaîne reste muette, derrière.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Mila revient vers la table. Le vent a touché le pain. Le seau, maman. Elle tire l'anse d'un coup. L'anse bute contre le pied. Il reste. Le manteau rouge bouge au dossier. Une manche tombe, large. Elle cache le clou de cuivre. On soulève tout ? Non. Mila refuse de foncer. Maman se met à sa hauteur. Personne ne dit le mot. Mila observe le seau, dans l'ombre. Elle écoute le bois. C'est l'heure, presque. Pas sans le toc. Le toc du clou. Tu l'as, ce son. La chaîne reste muette, derrière.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14760,6 +14779,8 @@
 narrateur|Personne ne dit le mot.
 narrateur|Mila observe le seau, dans l'ombre.
 narrateur|Elle écoute le bois.
+papa|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 enfant-f|Le toc du clou.
 maman|Tu l'as, ce son.
 narrateur|La chaîne reste muette, derrière.</t>
@@ -16127,17 +16148,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Près des balançoires, le doudou gris attend. Le tissu a pris le vent. Il cherche le seau, avec moi. Mila le serre contre sa joue. L'oreille grise cache l'ombre. Elle cherche l'anse, trop vite. Sa main trouve le banc de pierre. Pas lui. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. L'oreille du doudou est froide.</t>
+          <t>Près des balançoires, le doudou gris attend. Le tissu a pris le vent. Il cherche le seau, avec moi. Mila le serre contre sa joue. L'oreille grise cache l'ombre. Elle cherche l'anse, trop vite. Sa main trouve le banc de pierre. Pas lui. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. L'oreille du doudou est froide.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près des balançoires, le doudou gris attend. Le tissu a pris le vent. Il cherche le seau, avec moi. Mila le serre contre sa joue. L'oreille grise cache l'ombre. Elle cherche l'anse, trop vite. Sa main trouve le banc de pierre. Pas lui. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. L'oreille du doudou est froide.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Près des balançoires, le doudou gris attend. Le tissu a pris le vent. Il cherche le seau, avec moi. Mila le serre contre sa joue. L'oreille grise cache l'ombre. Elle cherche l'anse, trop vite. Sa main trouve le banc de pierre. Pas lui. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. L'oreille du doudou est froide.&lt;/prosody&gt;&lt;break time="540ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Près des balançoires, le doudou gris attend. Le tissu a pris le vent. Il cherche le seau, avec moi. Mila le serre contre sa joue. L'oreille grise cache l'ombre. Elle cherche l'anse, trop vite. Sa main trouve le banc de pierre. Pas lui. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. L'oreille du doudou est froide.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Près des balançoires, le doudou gris attend. Le tissu a pris le vent. Il cherche le seau, avec moi. Mila le serre contre sa joue. L'oreille grise cache l'ombre. Elle cherche l'anse, trop vite. Sa main trouve le banc de pierre. Pas lui. Le sourire de Mila reste bas. L'oreille, un peu de côté ? Papa se met à sa hauteur. J'attends. Mila refuse de foncer. Elle écarte l'oreille, lentement. C'est l'heure, presque. Pas sans le toc. Un toc minuscule, sous le bois. Le clou. Tu l'as entendu, seule. L'oreille du doudou est froide.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -16289,6 +16310,8 @@
 enfant-f|J'attends.
 narrateur|Mila refuse de foncer.
 narrateur|Elle écarte l'oreille, lentement.
+papa|C'est l'heure, presque.
+enfant-f|Pas sans le toc.
 narrateur|Un toc minuscule, sous le bois.
 enfant-f|Le clou.
 maman|Tu l'as entendu, seule.
@@ -17645,7 +17668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17758,6 +17781,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>